<commit_message>
Concorrentes por destino (Peterle, La Sofia, Pedra d'Agua), planilhas no formato do template e correcao de dois quadros
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-objetivos-smart.xlsx
+++ b/02-objetivos-smart.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template de Objetivos SMART" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objetivo 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objetivo 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objetivo 3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,14 +29,25 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font/>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5D3A"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -54,12 +67,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -427,242 +447,512 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="B2:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>OBJETIVOS SMART</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr"/>
-      <c r="C1" s="1" t="inlineStr"/>
-      <c r="D1" s="1" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Pousada Vila Mathilde (Matilde, Alfredo Chaves, ES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Período</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>6 meses a partir da aprovação do plano</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Desafio</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Aumentar as vendas e melhorar a imagem da marca, atraindo aposentados que buscam sossego e convertendo o visitante de excursão em hóspede.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Que ação específica norteará seu objetivo?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Corrigir bio do Instagram, Google Perfil da Empresa, telefone, WhatsApp Business e dados nas OTAs (café da manhã, número de quartos, check-in, fotos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1"/>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Como o objetivo será mensurado?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Checklist de 100% dos canais corrigidos e nenhuma avaliação nova reclamando de contato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1"/>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Esse objetivo é alcançável? Justifique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Sim. Depende de ajustes cadastrais, não de verba, e o dono tem acesso aos canais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1"/>
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Porque esse objetivo é relevante para a empresa?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Hoje o anúncio leva a canais que sinalizam "à venda" e "fechada". Sem isso, nenhuma mídia converte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1"/>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Em que prazo ele deve ser alcançado?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>30 dias</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1"/>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Redação final do Objetivo SMART</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Corrigir 100% dos pontos de contato digitais da pousada (Instagram, Google, WhatsApp e OTAs) em até 30 dias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="B12:E13"/>
+    <mergeCell ref="B8:E9"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B16:E17"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B20:E21"/>
+    <mergeCell ref="B28:E29"/>
+    <mergeCell ref="B24:E25"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:E29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>OBJETIVOS SMART</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Pousada Vila Mathilde (Matilde, Alfredo Chaves, ES)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>6 meses a partir da aprovação do plano</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Desafio</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Aumentar as vendas e melhorar a imagem da marca, atraindo aposentados que buscam sossego e convertendo o visitante de excursão em hóspede.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Que ação específica norteará seu objetivo?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Criar o pacote "Sossego de Meio de Semana" (domingo a quinta) para aposentados, divulgado em Reels, TikTok, vídeos no Facebook e WhatsApp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1"/>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Como o objetivo será mensurado?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Diárias vendidas de domingo a quinta por mês e taxa de ocupação nesses dias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1"/>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Esse objetivo é alcançável? Justifique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Sim. Aposentado tem flexibilidade de datas e esses dias hoje estão vazios, então não concorrem com o fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1"/>
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Porque esse objetivo é relevante para a empresa?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>O problema real é o vale entre os picos. Preencher dias ociosos gera receita sem investir em estrutura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1"/>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Em que prazo ele deve ser alcançado?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>6 meses</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1"/>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Redação final do Objetivo SMART</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Alcançar 40% de ocupação média de domingo a quinta em 6 meses, a partir do pacote Sossego de Meio de Semana. (Meta a calibrar com o histórico real.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="B12:E13"/>
+    <mergeCell ref="B8:E9"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B16:E17"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B20:E21"/>
+    <mergeCell ref="B28:E29"/>
+    <mergeCell ref="B24:E25"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:E29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>OBJETIVOS SMART</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Pousada Vila Mathilde (Matilde, Alfredo Chaves, ES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Período</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>6 meses a partir da aprovação do plano</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Desafio</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Aumentar as vendas e melhorar a imagem da marca, atraindo aposentados que buscam sossego e convertendo o visitante de excursão em hóspede.</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Pergunta</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Objetivo 1</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>Objetivo 2</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Objetivo 3</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Que ação específica norteará seu objetivo?</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Corrigir bio do Instagram, Google Perfil da Empresa, telefone, WhatsApp Business e dados nas OTAs.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Criar o pacote "Sossego de Meio de Semana" (domingo a quinta) para aposentados, divulgado em Reels, TikTok, vídeos no Facebook e WhatsApp.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Montar lista de contatos no WhatsApp (ex-hóspedes, indicações e visitantes de excursão) e enviar mensagem quinzenal com datas livres e tarifa direta.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9" ht="34" customHeight="1"/>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Como o objetivo será mensurado?</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Checklist de 100% dos canais corrigidos e nenhuma avaliação nova reclamando de contato.</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Diárias vendidas de domingo a quinta por mês e taxa de ocupação nesses dias.</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Tamanho da lista, reservas fechadas pelo WhatsApp e % de reservas diretas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Tamanho da lista, reservas fechadas pelo WhatsApp e % de reservas diretas sobre o total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1"/>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Esse objetivo é alcançável? Justifique.</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Sim. Depende de ajustes cadastrais, não de verba, e o dono tem acesso aos canais.</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sim. Aposentado tem flexibilidade de datas e esses dias hoje estão vazios.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Sim. Hóspedes elogiam o atendimento e o canal exige tempo, não verba.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Por que esse objetivo é relevante para a empresa?</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Hoje o anúncio leva a canais que sinalizam "à venda" e "fechada". Sem isso, nenhuma mídia converte.</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>O problema real é o vale entre os picos. Preencher dias ociosos gera receita sem investir em estrutura.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Evita comissão de 15% a 25% das OTAs e o idoso prefere falar com uma pessoa antes de reservar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="17" ht="34" customHeight="1"/>
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Porque esse objetivo é relevante para a empresa?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Evita comissão de 15% a 25% das OTAs e o público idoso prefere falar com uma pessoa antes de reservar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1"/>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Em que prazo ele deve ser alcançado?</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>30 dias</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>6 meses</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>6 meses</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    </row>
+    <row r="25" ht="34" customHeight="1"/>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Redação final do Objetivo SMART</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Corrigir 100% dos pontos de contato digitais da pousada (Instagram, Google, WhatsApp e OTAs) em até 30 dias.</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Alcançar 40% de ocupação média de domingo a quinta em 6 meses, a partir do pacote Sossego de Meio de Semana.</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Formar uma lista de 300 contatos no WhatsApp e chegar a 50% das reservas por venda direta em 6 meses.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Observação</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Metas de ocupação e vendas diretas a calibrar com o histórico real da pousada.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Formar uma lista de 300 contatos no WhatsApp e chegar a 50% das reservas por venda direta em 6 meses. (Metas a calibrar com o histórico.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1"/>
   </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="B12:E13"/>
+    <mergeCell ref="B8:E9"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B16:E17"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B20:E21"/>
+    <mergeCell ref="B28:E29"/>
+    <mergeCell ref="B24:E25"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>